<commit_message>
Fix demo-admin delete flow
</commit_message>
<xml_diff>
--- a/docs/仕様書.xlsx
+++ b/docs/仕様書.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\source\repos2\selfdrinkbar-system\docs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\source\repos2\membership-management-system\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{00EF1BE4-ED2C-4E42-949E-B6BBEA2D517D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9ABA6045-5E22-494E-A73C-7B776B97382B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-25545" yWindow="255" windowWidth="23505" windowHeight="13335" firstSheet="4" activeTab="6" xr2:uid="{B2A7CC7D-9061-4016-B10F-12143085F4DA}"/>
+    <workbookView xWindow="-25545" yWindow="255" windowWidth="23505" windowHeight="13335" firstSheet="3" activeTab="7" xr2:uid="{B2A7CC7D-9061-4016-B10F-12143085F4DA}"/>
   </bookViews>
   <sheets>
     <sheet name="01_システム概要" sheetId="1" r:id="rId1"/>
@@ -775,6 +775,889 @@
     <phoneticPr fontId="1"/>
   </si>
   <si>
+    <t>会員登録、ログイン、会員情報管理、管理者による検索・編集・削除、CSV入出力、メール送信、入力の際のバリデーション、パスワード変更・リセット</t>
+    <rPh sb="45" eb="47">
+      <t>ニュウリョク</t>
+    </rPh>
+    <rPh sb="48" eb="49">
+      <t>サイ</t>
+    </rPh>
+    <rPh sb="63" eb="65">
+      <t>ヘンコウ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>/admin/users/im_ex_port</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>CSVインポート・エクスポート画面</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>編集画面</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>メールにリセットページへのURL添付</t>
+    <rPh sb="16" eb="18">
+      <t>テンプ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>会員一覧画面</t>
+    <rPh sb="0" eb="2">
+      <t>カイイン</t>
+    </rPh>
+    <rPh sb="2" eb="4">
+      <t>イチラン</t>
+    </rPh>
+    <rPh sb="4" eb="6">
+      <t>ガメン</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>管理者画面画面、会員一覧画面</t>
+    <rPh sb="3" eb="5">
+      <t>ガメン</t>
+    </rPh>
+    <rPh sb="5" eb="7">
+      <t>ガメン</t>
+    </rPh>
+    <rPh sb="8" eb="14">
+      <t>カイインイチランガメン</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>会員一覧画面</t>
+    <rPh sb="0" eb="6">
+      <t>カイインイチランガメン</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>会員詳細画面、会員詳細編集画面</t>
+    <rPh sb="0" eb="2">
+      <t>カイイン</t>
+    </rPh>
+    <rPh sb="2" eb="4">
+      <t>ショウサイ</t>
+    </rPh>
+    <rPh sb="4" eb="6">
+      <t>ガメン</t>
+    </rPh>
+    <rPh sb="7" eb="9">
+      <t>カイイン</t>
+    </rPh>
+    <rPh sb="9" eb="11">
+      <t>ショウサイ</t>
+    </rPh>
+    <rPh sb="11" eb="13">
+      <t>ヘンシュウ</t>
+    </rPh>
+    <rPh sb="13" eb="15">
+      <t>ガメン</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>会員詳細画面</t>
+    <rPh sb="0" eb="2">
+      <t>カイイン</t>
+    </rPh>
+    <rPh sb="2" eb="4">
+      <t>ショウサイ</t>
+    </rPh>
+    <rPh sb="4" eb="6">
+      <t>ガメン</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>super→superとadmin01のパスワード変更、admin01→admin01のパスワード変更</t>
+    <rPh sb="25" eb="27">
+      <t>ヘンコウ</t>
+    </rPh>
+    <rPh sb="49" eb="51">
+      <t>ヘンコウ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>管理者・上位管理者</t>
+    <rPh sb="0" eb="3">
+      <t>カンリシャ</t>
+    </rPh>
+    <rPh sb="4" eb="9">
+      <t>ジョウイカンリシャ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>会員</t>
+    <rPh sb="0" eb="2">
+      <t>カイイン</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>会員・管理者</t>
+    <rPh sb="0" eb="2">
+      <t>カイイン</t>
+    </rPh>
+    <rPh sb="3" eb="6">
+      <t>カンリシャ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>退会者削除</t>
+    <rPh sb="0" eb="3">
+      <t>タイカイシャ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>zipcloud(API)</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>パスワードを忘れたとき</t>
+    <rPh sb="6" eb="7">
+      <t>ワス</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>パスワードリセットURL送信メール</t>
+    <rPh sb="12" eb="14">
+      <t>ソウシン</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>あいうえお美術館会員登録完了のお知らせ</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>あいうえお美術館退会手続き完了のお知らせ</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>2. 退会完了メール</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>2. パスワードリセットメール</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>あいうえお美術館：パスワードリセット手続き</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>email, reset_url</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>zipcode</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>VARCHAR</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>郵便番号</t>
+    <rPh sb="0" eb="4">
+      <t>ユウビンバンゴウ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>活動中・休会中・退会</t>
+    <rPh sb="0" eb="3">
+      <t>カツドウチュウ</t>
+    </rPh>
+    <rPh sb="4" eb="7">
+      <t>キュウカイチュウ</t>
+    </rPh>
+    <rPh sb="8" eb="10">
+      <t>タイカイ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>username</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>管理者アカウント</t>
+    <rPh sb="0" eb="3">
+      <t>カンリシャ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>管理者・上位管理者</t>
+    <rPh sb="0" eb="3">
+      <t>カンリシャ</t>
+    </rPh>
+    <rPh sb="4" eb="6">
+      <t>ジョウイ</t>
+    </rPh>
+    <rPh sb="6" eb="9">
+      <t>カンリシャ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>mail_logsテーブル</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>user_id</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>mail_type</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>sent_at</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>INT</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>DATETIME</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>外部キー</t>
+    <rPh sb="0" eb="2">
+      <t>ガイブ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>更新日時</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>会員登録・退会・パスワードリセット</t>
+    <rPh sb="0" eb="4">
+      <t>カイイントウロク</t>
+    </rPh>
+    <rPh sb="5" eb="7">
+      <t>タイカイ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>ルート</t>
+  </si>
+  <si>
+    <t>入力</t>
+  </si>
+  <si>
+    <t>出力 / 遷移</t>
+  </si>
+  <si>
+    <t>TOP /</t>
+  </si>
+  <si>
+    <t>トップページ表示</t>
+  </si>
+  <si>
+    <t>index.html</t>
+  </si>
+  <si>
+    <t>会員登録 /register</t>
+  </si>
+  <si>
+    <t>GET / POST</t>
+  </si>
+  <si>
+    <t>会員登録フォーム表示・登録処理</t>
+  </si>
+  <si>
+    <t>name, email, zipcode, address, phone, password</t>
+  </si>
+  <si>
+    <t>成功→login 失敗→register 再表示</t>
+  </si>
+  <si>
+    <t>ログイン /login</t>
+  </si>
+  <si>
+    <t>ログイン処理</t>
+  </si>
+  <si>
+    <t>成功→mypage 失敗→login</t>
+  </si>
+  <si>
+    <t>ログアウト /logout</t>
+  </si>
+  <si>
+    <t>ログアウト処理</t>
+  </si>
+  <si>
+    <t>login.html</t>
+  </si>
+  <si>
+    <t>パスワードリセットメール送信</t>
+  </si>
+  <si>
+    <t>成功→login 失敗→forget_pw</t>
+  </si>
+  <si>
+    <t>新パスワード設定</t>
+  </si>
+  <si>
+    <t>password_new, password_check</t>
+  </si>
+  <si>
+    <t>成功→login 失敗→reset_password</t>
+  </si>
+  <si>
+    <t>パスワード忘れ /forget_pw</t>
+  </si>
+  <si>
+    <t>パスワード再設定 /reset_password/&lt;token&gt;</t>
+  </si>
+  <si>
+    <t>マイページ /mypage</t>
+  </si>
+  <si>
+    <t>mypage.html</t>
+  </si>
+  <si>
+    <t>会員情報編集 /mypage/edit</t>
+  </si>
+  <si>
+    <t>パスワード変更 /ch_password</t>
+  </si>
+  <si>
+    <t>パスワード変更</t>
+  </si>
+  <si>
+    <t>pw_current, pw_new, pw_check</t>
+  </si>
+  <si>
+    <t>成功→mypage 失敗→ch_password</t>
+  </si>
+  <si>
+    <t>1. validate_user_input（会員登録・会員編集・管理者編集で使用）</t>
+  </si>
+  <si>
+    <t>No</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>条件</t>
+  </si>
+  <si>
+    <t>エラーメッセージ</t>
+  </si>
+  <si>
+    <t>適用</t>
+  </si>
+  <si>
+    <t>名前必須</t>
+  </si>
+  <si>
+    <t>name が空</t>
+  </si>
+  <si>
+    <t>名前・メールは必須です</t>
+  </si>
+  <si>
+    <t>register / edit</t>
+  </si>
+  <si>
+    <t>メール必須</t>
+  </si>
+  <si>
+    <t>email が空</t>
+  </si>
+  <si>
+    <t>正規表現不一致</t>
+  </si>
+  <si>
+    <t>メールアドレスの形式が正しくありません</t>
+  </si>
+  <si>
+    <t>全画面</t>
+  </si>
+  <si>
+    <t>メール重複</t>
+  </si>
+  <si>
+    <t>同じ email が既に存在（current_user_id を除く）</t>
+  </si>
+  <si>
+    <t>このメールアドレスは既に登録されています</t>
+  </si>
+  <si>
+    <t>郵便番号必須</t>
+  </si>
+  <si>
+    <t>zipcode が空</t>
+  </si>
+  <si>
+    <t>郵便番号を入力してください</t>
+  </si>
+  <si>
+    <t>7桁チェック</t>
+  </si>
+  <si>
+    <t>数字でない or 7桁でない</t>
+  </si>
+  <si>
+    <t>郵便番号は7桁の数字で入力してください</t>
+  </si>
+  <si>
+    <t>存在チェック（API）</t>
+  </si>
+  <si>
+    <t>zipcloud API の results が None</t>
+  </si>
+  <si>
+    <t>存在しない郵便番号です</t>
+  </si>
+  <si>
+    <t>住所必須</t>
+  </si>
+  <si>
+    <t>address が空</t>
+  </si>
+  <si>
+    <t>住所が空欄です。郵便番号を入れて検索ボタンを押してください</t>
+  </si>
+  <si>
+    <t>住所長さ</t>
+  </si>
+  <si>
+    <t>200文字超</t>
+  </si>
+  <si>
+    <t>住所が長すぎます</t>
+  </si>
+  <si>
+    <t>パスワード必須</t>
+  </si>
+  <si>
+    <t>password が空</t>
+  </si>
+  <si>
+    <t>パスワードは必須です</t>
+  </si>
+  <si>
+    <t>register</t>
+  </si>
+  <si>
+    <t>パスワード強度</t>
+  </si>
+  <si>
+    <t>3文字未満</t>
+  </si>
+  <si>
+    <t>パスワードは3文字以上で入力してください</t>
+  </si>
+  <si>
+    <t>register / reset</t>
+  </si>
+  <si>
+    <t>パスワード一致</t>
+  </si>
+  <si>
+    <t>password ≠ password_check</t>
+  </si>
+  <si>
+    <t>新しいパスワードが一致しません</t>
+  </si>
+  <si>
+    <t>数字チェック</t>
+  </si>
+  <si>
+    <t>ハイフン除去後に数字以外が含まれる</t>
+  </si>
+  <si>
+    <t>電話番号は数字とハイフンのみで入力してください</t>
+  </si>
+  <si>
+    <t>桁数チェック</t>
+  </si>
+  <si>
+    <t>10〜11桁以外</t>
+  </si>
+  <si>
+    <t>電話番号は10桁または11桁で入力してください</t>
+  </si>
+  <si>
+    <t>空欄は許可</t>
+  </si>
+  <si>
+    <t>phone が空</t>
+  </si>
+  <si>
+    <t>チェックなし</t>
+  </si>
+  <si>
+    <t>2. validate_user_pw_input（パスワード変更・管理者パスワード変更）</t>
+  </si>
+  <si>
+    <t>現行パスワード一致</t>
+  </si>
+  <si>
+    <t>check_password_hash が False</t>
+  </si>
+  <si>
+    <t>現在のパスワードが正しくありません</t>
+  </si>
+  <si>
+    <t>ch_password / ch_admins_password</t>
+  </si>
+  <si>
+    <t>新パスワード一致</t>
+  </si>
+  <si>
+    <t>pw_new ≠ pw_check</t>
+  </si>
+  <si>
+    <t>pw_new が 3文字未満</t>
+  </si>
+  <si>
+    <t>現行と同じ禁止</t>
+  </si>
+  <si>
+    <t>pw_new が現行と同じ</t>
+  </si>
+  <si>
+    <t>新しいパスワードが現在のパスワードと同じです</t>
+  </si>
+  <si>
+    <t>■基本情報チェック</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>■電話番号チェック（任意入力）</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>■パスワードチェック（新規登録・パスワード変更）</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>■郵便番号チェック（zipcloud API 使用）</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>■パスワード変更用バリデーション</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>休会 /inactive</t>
+    <rPh sb="0" eb="2">
+      <t>キュウカイ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>POST</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>休会</t>
+    <rPh sb="0" eb="2">
+      <t>キュウカイ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>再開 /reactivate</t>
+    <rPh sb="0" eb="2">
+      <t>サイカイ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>会員情報編集</t>
+    <rPh sb="4" eb="6">
+      <t>ヘンシュウ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>name, email, zipcode, address, phone</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>mypage_edit.html</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>退会 /withdraw</t>
+    <rPh sb="0" eb="2">
+      <t>タイカイ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>再開</t>
+    <rPh sb="0" eb="2">
+      <t>サイカイ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>退会</t>
+    <rPh sb="0" eb="2">
+      <t>タイカイ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>login.html</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>ログアウト /logout</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>GET</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>管理者ログイン /admin_login</t>
+    <rPh sb="0" eb="3">
+      <t>カンリシャ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>管理者ログイン</t>
+    <rPh sb="0" eb="3">
+      <t>カンリシャ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>username,password</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>成功→admin_search_form 失敗→admin_login</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>会員検索フォーム表示 /admin/search</t>
+    <rPh sb="0" eb="4">
+      <t>カイインケンサク</t>
+    </rPh>
+    <rPh sb="8" eb="10">
+      <t>ヒョウジ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>会員検索フォーム表示</t>
+    <rPh sb="0" eb="4">
+      <t>カイインケンサク</t>
+    </rPh>
+    <rPh sb="8" eb="10">
+      <t>ヒョウジ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>admin/search.html</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>会員検索 /admin/search/results</t>
+    <rPh sb="0" eb="4">
+      <t>カイインケンサク</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>GET / POST</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>会員検索</t>
+    <rPh sb="0" eb="4">
+      <t>カイインケンサク</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>name,email,address,status</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>admin/users.html</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>会員詳細 /admin/users/&lt;int:id&gt;</t>
+    <rPh sb="0" eb="4">
+      <t>カイインショウサイ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>会員詳細</t>
+    <rPh sb="0" eb="4">
+      <t>カイインショウサイ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>admin/user_detail.html</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>会員編集 /admin/users/edit/&lt;int:id&gt;</t>
+    <rPh sb="0" eb="4">
+      <t>カイインヘンシュウ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>会員編集</t>
+    <rPh sb="0" eb="4">
+      <t>カイインヘンシュウ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>admin/user_detail_edit.html</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>会員削除 /admin/users/delete/&lt;int:id&gt;</t>
+    <rPh sb="0" eb="2">
+      <t>カイイン</t>
+    </rPh>
+    <rPh sb="2" eb="4">
+      <t>サクジョ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>会員削除</t>
+    <rPh sb="0" eb="4">
+      <t>カイインサクジョ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>成功→admin_search_form 失敗→user_detail.html</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>管理者パスワード変更 /ch_admins_password</t>
+    <rPh sb="0" eb="3">
+      <t>カンリシャ</t>
+    </rPh>
+    <rPh sb="8" eb="10">
+      <t>ヘンコウ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>成功→admin_search_form 失敗→admin/search.html</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>管理者ログアウト /admin/logout</t>
+    <rPh sb="0" eb="3">
+      <t>カンリシャ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>管理者ログアウト</t>
+    <rPh sb="0" eb="3">
+      <t>カンリシャ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>admin/login.html</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>CSVインポート・エクスポート /admin/users/in_ex_port</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>CSVインポート・エクスポート画面</t>
+    <rPh sb="15" eb="17">
+      <t>ガメン</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>admin/users/im_ex_port.html</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>CSVインポート /admin/users/import</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>CSVインポート</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>成功→admin/im_ex_port.html 失敗→admin/search_form</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>CSVエクスポート /admin/user/export</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>CSVエクスポート</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>{{ user.name }}様
+この度は、あいうえお美術館の会員登録をいただき、誠に有難うございます。
+以下の内容でユーザー登録が完了しました。
+~~~~~~~~~~~~~~~~~~~~~~~~~~~~~~~~
+■登録情報
+お名前：{{ user.name }}
+メールアドレス：{{ user.email }}
+登録日時：{{ user.created_at }}
+~~~~~~~~~~~~~~~~~~~~~~~~~~~~~~~~
+今後とも当館を宜しくお願い致します。
+あいうえお美術館会員管理システム
+noreply@oestemar-portfolio.xyz</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>{{ email }}様
+あいうえお美術館のパスワードリセット手続きは下記リンクを開いて進めてください。
+◆パスワードリセットURL
+{{ reset_url }}
+※1時間以内にパスワード更新作業を完了しないとキャンセルとなります。
+あいうえお美術館会員管理システム
+noreply@oestemar-portfolio.xyz</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
     <t>{{ user.name }}様
 この度は、あいうえお美術館の会員退会手続きを承りました。
 以下の内容で退会処理が完了しました。
@@ -786,890 +1669,7 @@
 これまでご利用いただき、誠に有難うございました。
 またのご利用を心よりお待ちしております。
 あいうえお美術館会員管理システム
-noreply.aiueosystem@gmail.com</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>{{ user.name }}様
-この度は、あいうえお美術館の会員登録をいただき、誠に有難うございます。
-以下の内容でユーザー登録が完了しました。
-~~~~~~~~~~~~~~~~~~~~~~~~~~~~~~~~
-■登録情報
-お名前：{{ user.name }}
-メールアドレス：{{ user.email }}
-登録日時：{{ user.created_at }}
-~~~~~~~~~~~~~~~~~~~~~~~~~~~~~~~~
-今後とも当館を宜しくお願い致します。
-あいうえお美術館会員管理システム
-noreply.aiueosystem@gmail.com</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>会員登録、ログイン、会員情報管理、管理者による検索・編集・削除、CSV入出力、メール送信、入力の際のバリデーション、パスワード変更・リセット</t>
-    <rPh sb="45" eb="47">
-      <t>ニュウリョク</t>
-    </rPh>
-    <rPh sb="48" eb="49">
-      <t>サイ</t>
-    </rPh>
-    <rPh sb="63" eb="65">
-      <t>ヘンコウ</t>
-    </rPh>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>/admin/users/im_ex_port</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>CSVインポート・エクスポート画面</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>編集画面</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>メールにリセットページへのURL添付</t>
-    <rPh sb="16" eb="18">
-      <t>テンプ</t>
-    </rPh>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>会員一覧画面</t>
-    <rPh sb="0" eb="2">
-      <t>カイイン</t>
-    </rPh>
-    <rPh sb="2" eb="4">
-      <t>イチラン</t>
-    </rPh>
-    <rPh sb="4" eb="6">
-      <t>ガメン</t>
-    </rPh>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>管理者画面画面、会員一覧画面</t>
-    <rPh sb="3" eb="5">
-      <t>ガメン</t>
-    </rPh>
-    <rPh sb="5" eb="7">
-      <t>ガメン</t>
-    </rPh>
-    <rPh sb="8" eb="14">
-      <t>カイインイチランガメン</t>
-    </rPh>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>会員一覧画面</t>
-    <rPh sb="0" eb="6">
-      <t>カイインイチランガメン</t>
-    </rPh>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>会員詳細画面、会員詳細編集画面</t>
-    <rPh sb="0" eb="2">
-      <t>カイイン</t>
-    </rPh>
-    <rPh sb="2" eb="4">
-      <t>ショウサイ</t>
-    </rPh>
-    <rPh sb="4" eb="6">
-      <t>ガメン</t>
-    </rPh>
-    <rPh sb="7" eb="9">
-      <t>カイイン</t>
-    </rPh>
-    <rPh sb="9" eb="11">
-      <t>ショウサイ</t>
-    </rPh>
-    <rPh sb="11" eb="13">
-      <t>ヘンシュウ</t>
-    </rPh>
-    <rPh sb="13" eb="15">
-      <t>ガメン</t>
-    </rPh>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>会員詳細画面</t>
-    <rPh sb="0" eb="2">
-      <t>カイイン</t>
-    </rPh>
-    <rPh sb="2" eb="4">
-      <t>ショウサイ</t>
-    </rPh>
-    <rPh sb="4" eb="6">
-      <t>ガメン</t>
-    </rPh>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>super→superとadmin01のパスワード変更、admin01→admin01のパスワード変更</t>
-    <rPh sb="25" eb="27">
-      <t>ヘンコウ</t>
-    </rPh>
-    <rPh sb="49" eb="51">
-      <t>ヘンコウ</t>
-    </rPh>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>管理者・上位管理者</t>
-    <rPh sb="0" eb="3">
-      <t>カンリシャ</t>
-    </rPh>
-    <rPh sb="4" eb="9">
-      <t>ジョウイカンリシャ</t>
-    </rPh>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>会員</t>
-    <rPh sb="0" eb="2">
-      <t>カイイン</t>
-    </rPh>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>会員・管理者</t>
-    <rPh sb="0" eb="2">
-      <t>カイイン</t>
-    </rPh>
-    <rPh sb="3" eb="6">
-      <t>カンリシャ</t>
-    </rPh>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>退会者削除</t>
-    <rPh sb="0" eb="3">
-      <t>タイカイシャ</t>
-    </rPh>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>zipcloud(API)</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>パスワードを忘れたとき</t>
-    <rPh sb="6" eb="7">
-      <t>ワス</t>
-    </rPh>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>パスワードリセットURL送信メール</t>
-    <rPh sb="12" eb="14">
-      <t>ソウシン</t>
-    </rPh>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>あいうえお美術館会員登録完了のお知らせ</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>あいうえお美術館退会手続き完了のお知らせ</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>2. 退会完了メール</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>2. パスワードリセットメール</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>あいうえお美術館：パスワードリセット手続き</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>{{ email }}様
-あいうえお美術館のパスワードリセット手続きは下記リンクを開いて進めてください。
-◆パスワードリセットURL
-{{ reset_url }}
-※1時間以内にパスワード更新作業を完了しないとキャンセルとなります。
-あいうえお美術館会員管理システム
-noreply.aiueosystem@gmail.com</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>email, reset_url</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>zipcode</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>VARCHAR</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>郵便番号</t>
-    <rPh sb="0" eb="4">
-      <t>ユウビンバンゴウ</t>
-    </rPh>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>活動中・休会中・退会</t>
-    <rPh sb="0" eb="3">
-      <t>カツドウチュウ</t>
-    </rPh>
-    <rPh sb="4" eb="7">
-      <t>キュウカイチュウ</t>
-    </rPh>
-    <rPh sb="8" eb="10">
-      <t>タイカイ</t>
-    </rPh>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>username</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>管理者アカウント</t>
-    <rPh sb="0" eb="3">
-      <t>カンリシャ</t>
-    </rPh>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>管理者・上位管理者</t>
-    <rPh sb="0" eb="3">
-      <t>カンリシャ</t>
-    </rPh>
-    <rPh sb="4" eb="6">
-      <t>ジョウイ</t>
-    </rPh>
-    <rPh sb="6" eb="9">
-      <t>カンリシャ</t>
-    </rPh>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>mail_logsテーブル</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>user_id</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>mail_type</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>sent_at</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>INT</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>DATETIME</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>外部キー</t>
-    <rPh sb="0" eb="2">
-      <t>ガイブ</t>
-    </rPh>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>更新日時</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>会員登録・退会・パスワードリセット</t>
-    <rPh sb="0" eb="4">
-      <t>カイイントウロク</t>
-    </rPh>
-    <rPh sb="5" eb="7">
-      <t>タイカイ</t>
-    </rPh>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>ルート</t>
-  </si>
-  <si>
-    <t>入力</t>
-  </si>
-  <si>
-    <t>出力 / 遷移</t>
-  </si>
-  <si>
-    <t>TOP /</t>
-  </si>
-  <si>
-    <t>トップページ表示</t>
-  </si>
-  <si>
-    <t>index.html</t>
-  </si>
-  <si>
-    <t>会員登録 /register</t>
-  </si>
-  <si>
-    <t>GET / POST</t>
-  </si>
-  <si>
-    <t>会員登録フォーム表示・登録処理</t>
-  </si>
-  <si>
-    <t>name, email, zipcode, address, phone, password</t>
-  </si>
-  <si>
-    <t>成功→login 失敗→register 再表示</t>
-  </si>
-  <si>
-    <t>ログイン /login</t>
-  </si>
-  <si>
-    <t>ログイン処理</t>
-  </si>
-  <si>
-    <t>成功→mypage 失敗→login</t>
-  </si>
-  <si>
-    <t>ログアウト /logout</t>
-  </si>
-  <si>
-    <t>ログアウト処理</t>
-  </si>
-  <si>
-    <t>login.html</t>
-  </si>
-  <si>
-    <t>パスワードリセットメール送信</t>
-  </si>
-  <si>
-    <t>成功→login 失敗→forget_pw</t>
-  </si>
-  <si>
-    <t>新パスワード設定</t>
-  </si>
-  <si>
-    <t>password_new, password_check</t>
-  </si>
-  <si>
-    <t>成功→login 失敗→reset_password</t>
-  </si>
-  <si>
-    <t>パスワード忘れ /forget_pw</t>
-  </si>
-  <si>
-    <t>パスワード再設定 /reset_password/&lt;token&gt;</t>
-  </si>
-  <si>
-    <t>マイページ /mypage</t>
-  </si>
-  <si>
-    <t>mypage.html</t>
-  </si>
-  <si>
-    <t>会員情報編集 /mypage/edit</t>
-  </si>
-  <si>
-    <t>パスワード変更 /ch_password</t>
-  </si>
-  <si>
-    <t>パスワード変更</t>
-  </si>
-  <si>
-    <t>pw_current, pw_new, pw_check</t>
-  </si>
-  <si>
-    <t>成功→mypage 失敗→ch_password</t>
-  </si>
-  <si>
-    <t>1. validate_user_input（会員登録・会員編集・管理者編集で使用）</t>
-  </si>
-  <si>
-    <t>No</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>条件</t>
-  </si>
-  <si>
-    <t>エラーメッセージ</t>
-  </si>
-  <si>
-    <t>適用</t>
-  </si>
-  <si>
-    <t>名前必須</t>
-  </si>
-  <si>
-    <t>name が空</t>
-  </si>
-  <si>
-    <t>名前・メールは必須です</t>
-  </si>
-  <si>
-    <t>register / edit</t>
-  </si>
-  <si>
-    <t>メール必須</t>
-  </si>
-  <si>
-    <t>email が空</t>
-  </si>
-  <si>
-    <t>正規表現不一致</t>
-  </si>
-  <si>
-    <t>メールアドレスの形式が正しくありません</t>
-  </si>
-  <si>
-    <t>全画面</t>
-  </si>
-  <si>
-    <t>メール重複</t>
-  </si>
-  <si>
-    <t>同じ email が既に存在（current_user_id を除く）</t>
-  </si>
-  <si>
-    <t>このメールアドレスは既に登録されています</t>
-  </si>
-  <si>
-    <t>郵便番号必須</t>
-  </si>
-  <si>
-    <t>zipcode が空</t>
-  </si>
-  <si>
-    <t>郵便番号を入力してください</t>
-  </si>
-  <si>
-    <t>7桁チェック</t>
-  </si>
-  <si>
-    <t>数字でない or 7桁でない</t>
-  </si>
-  <si>
-    <t>郵便番号は7桁の数字で入力してください</t>
-  </si>
-  <si>
-    <t>存在チェック（API）</t>
-  </si>
-  <si>
-    <t>zipcloud API の results が None</t>
-  </si>
-  <si>
-    <t>存在しない郵便番号です</t>
-  </si>
-  <si>
-    <t>住所必須</t>
-  </si>
-  <si>
-    <t>address が空</t>
-  </si>
-  <si>
-    <t>住所が空欄です。郵便番号を入れて検索ボタンを押してください</t>
-  </si>
-  <si>
-    <t>住所長さ</t>
-  </si>
-  <si>
-    <t>200文字超</t>
-  </si>
-  <si>
-    <t>住所が長すぎます</t>
-  </si>
-  <si>
-    <t>パスワード必須</t>
-  </si>
-  <si>
-    <t>password が空</t>
-  </si>
-  <si>
-    <t>パスワードは必須です</t>
-  </si>
-  <si>
-    <t>register</t>
-  </si>
-  <si>
-    <t>パスワード強度</t>
-  </si>
-  <si>
-    <t>3文字未満</t>
-  </si>
-  <si>
-    <t>パスワードは3文字以上で入力してください</t>
-  </si>
-  <si>
-    <t>register / reset</t>
-  </si>
-  <si>
-    <t>パスワード一致</t>
-  </si>
-  <si>
-    <t>password ≠ password_check</t>
-  </si>
-  <si>
-    <t>新しいパスワードが一致しません</t>
-  </si>
-  <si>
-    <t>数字チェック</t>
-  </si>
-  <si>
-    <t>ハイフン除去後に数字以外が含まれる</t>
-  </si>
-  <si>
-    <t>電話番号は数字とハイフンのみで入力してください</t>
-  </si>
-  <si>
-    <t>桁数チェック</t>
-  </si>
-  <si>
-    <t>10〜11桁以外</t>
-  </si>
-  <si>
-    <t>電話番号は10桁または11桁で入力してください</t>
-  </si>
-  <si>
-    <t>空欄は許可</t>
-  </si>
-  <si>
-    <t>phone が空</t>
-  </si>
-  <si>
-    <t>チェックなし</t>
-  </si>
-  <si>
-    <t>2. validate_user_pw_input（パスワード変更・管理者パスワード変更）</t>
-  </si>
-  <si>
-    <t>現行パスワード一致</t>
-  </si>
-  <si>
-    <t>check_password_hash が False</t>
-  </si>
-  <si>
-    <t>現在のパスワードが正しくありません</t>
-  </si>
-  <si>
-    <t>ch_password / ch_admins_password</t>
-  </si>
-  <si>
-    <t>新パスワード一致</t>
-  </si>
-  <si>
-    <t>pw_new ≠ pw_check</t>
-  </si>
-  <si>
-    <t>pw_new が 3文字未満</t>
-  </si>
-  <si>
-    <t>現行と同じ禁止</t>
-  </si>
-  <si>
-    <t>pw_new が現行と同じ</t>
-  </si>
-  <si>
-    <t>新しいパスワードが現在のパスワードと同じです</t>
-  </si>
-  <si>
-    <t>■基本情報チェック</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>■電話番号チェック（任意入力）</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>■パスワードチェック（新規登録・パスワード変更）</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>■郵便番号チェック（zipcloud API 使用）</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>■パスワード変更用バリデーション</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>休会 /inactive</t>
-    <rPh sb="0" eb="2">
-      <t>キュウカイ</t>
-    </rPh>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>POST</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>休会</t>
-    <rPh sb="0" eb="2">
-      <t>キュウカイ</t>
-    </rPh>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>再開 /reactivate</t>
-    <rPh sb="0" eb="2">
-      <t>サイカイ</t>
-    </rPh>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>会員情報編集</t>
-    <rPh sb="4" eb="6">
-      <t>ヘンシュウ</t>
-    </rPh>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>name, email, zipcode, address, phone</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>mypage_edit.html</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>退会 /withdraw</t>
-    <rPh sb="0" eb="2">
-      <t>タイカイ</t>
-    </rPh>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>再開</t>
-    <rPh sb="0" eb="2">
-      <t>サイカイ</t>
-    </rPh>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>退会</t>
-    <rPh sb="0" eb="2">
-      <t>タイカイ</t>
-    </rPh>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>login.html</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>ログアウト /logout</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>GET</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>管理者ログイン /admin_login</t>
-    <rPh sb="0" eb="3">
-      <t>カンリシャ</t>
-    </rPh>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>管理者ログイン</t>
-    <rPh sb="0" eb="3">
-      <t>カンリシャ</t>
-    </rPh>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>username,password</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>成功→admin_search_form 失敗→admin_login</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>会員検索フォーム表示 /admin/search</t>
-    <rPh sb="0" eb="4">
-      <t>カイインケンサク</t>
-    </rPh>
-    <rPh sb="8" eb="10">
-      <t>ヒョウジ</t>
-    </rPh>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>会員検索フォーム表示</t>
-    <rPh sb="0" eb="4">
-      <t>カイインケンサク</t>
-    </rPh>
-    <rPh sb="8" eb="10">
-      <t>ヒョウジ</t>
-    </rPh>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>admin/search.html</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>会員検索 /admin/search/results</t>
-    <rPh sb="0" eb="4">
-      <t>カイインケンサク</t>
-    </rPh>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>GET / POST</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>会員検索</t>
-    <rPh sb="0" eb="4">
-      <t>カイインケンサク</t>
-    </rPh>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>name,email,address,status</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>admin/users.html</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>会員詳細 /admin/users/&lt;int:id&gt;</t>
-    <rPh sb="0" eb="4">
-      <t>カイインショウサイ</t>
-    </rPh>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>会員詳細</t>
-    <rPh sb="0" eb="4">
-      <t>カイインショウサイ</t>
-    </rPh>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>admin/user_detail.html</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>会員編集 /admin/users/edit/&lt;int:id&gt;</t>
-    <rPh sb="0" eb="4">
-      <t>カイインヘンシュウ</t>
-    </rPh>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>会員編集</t>
-    <rPh sb="0" eb="4">
-      <t>カイインヘンシュウ</t>
-    </rPh>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>admin/user_detail_edit.html</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>会員削除 /admin/users/delete/&lt;int:id&gt;</t>
-    <rPh sb="0" eb="2">
-      <t>カイイン</t>
-    </rPh>
-    <rPh sb="2" eb="4">
-      <t>サクジョ</t>
-    </rPh>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>会員削除</t>
-    <rPh sb="0" eb="4">
-      <t>カイインサクジョ</t>
-    </rPh>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>成功→admin_search_form 失敗→user_detail.html</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>管理者パスワード変更 /ch_admins_password</t>
-    <rPh sb="0" eb="3">
-      <t>カンリシャ</t>
-    </rPh>
-    <rPh sb="8" eb="10">
-      <t>ヘンコウ</t>
-    </rPh>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>成功→admin_search_form 失敗→admin/search.html</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>管理者ログアウト /admin/logout</t>
-    <rPh sb="0" eb="3">
-      <t>カンリシャ</t>
-    </rPh>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>管理者ログアウト</t>
-    <rPh sb="0" eb="3">
-      <t>カンリシャ</t>
-    </rPh>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>admin/login.html</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>CSVインポート・エクスポート /admin/users/in_ex_port</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>CSVインポート・エクスポート画面</t>
-    <rPh sb="15" eb="17">
-      <t>ガメン</t>
-    </rPh>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>admin/users/im_ex_port.html</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>CSVインポート /admin/users/import</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>CSVインポート</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>成功→admin/im_ex_port.html 失敗→admin/search_form</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>CSVエクスポート /admin/user/export</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>CSVエクスポート</t>
+noreply@oestemar-portfolio.xyz</t>
     <phoneticPr fontId="1"/>
   </si>
 </sst>
@@ -2135,7 +2135,7 @@
         <v>11</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.4">
@@ -2253,7 +2253,7 @@
         <v>31</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="F5" s="1" t="s">
         <v>144</v>
@@ -2273,7 +2273,7 @@
         <v>35</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="F6" s="1"/>
     </row>
@@ -2329,7 +2329,7 @@
         <v>160</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="F9" s="1"/>
     </row>
@@ -2365,7 +2365,7 @@
         <v>127</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="F11" s="1" t="s">
         <v>128</v>
@@ -2373,7 +2373,7 @@
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A12" s="1" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="B12" s="1" t="s">
         <v>126</v>
@@ -2385,7 +2385,7 @@
         <v>125</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="F12" s="1"/>
     </row>
@@ -2403,7 +2403,7 @@
         <v>125</v>
       </c>
       <c r="E13" s="1" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="F13" s="1" t="s">
         <v>43</v>
@@ -2423,7 +2423,7 @@
         <v>141</v>
       </c>
       <c r="E14" s="1" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="F14" s="1"/>
     </row>
@@ -2441,16 +2441,16 @@
         <v>125</v>
       </c>
       <c r="E15" s="1" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="F15" s="1"/>
     </row>
     <row r="16" spans="1:6" ht="45" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A16" s="2" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="C16" s="1" t="s">
         <v>44</v>
@@ -2459,7 +2459,7 @@
         <v>139</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="F16" s="1"/>
     </row>
@@ -2519,7 +2519,7 @@
         <v>48</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="D2" s="1" t="s">
         <v>49</v>
@@ -2533,7 +2533,7 @@
         <v>51</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="D3" s="1" t="s">
         <v>52</v>
@@ -2547,7 +2547,7 @@
         <v>53</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="D4" s="1"/>
     </row>
@@ -2559,7 +2559,7 @@
         <v>55</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="D5" s="1"/>
     </row>
@@ -2571,7 +2571,7 @@
         <v>57</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="D6" s="1" t="s">
         <v>49</v>
@@ -2585,7 +2585,7 @@
         <v>161</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="D7" s="1"/>
     </row>
@@ -2597,7 +2597,7 @@
         <v>163</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="D8" s="1" t="s">
         <v>165</v>
@@ -2653,7 +2653,7 @@
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A13" s="1" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="B13" s="1" t="s">
         <v>61</v>
@@ -2692,10 +2692,10 @@
         <v>147</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="D16" s="1"/>
     </row>
@@ -2730,7 +2730,7 @@
         <v>154</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="C19" s="1" t="s">
         <v>153</v>
@@ -2967,10 +2967,10 @@
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A4" s="1" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>70</v>
@@ -2993,7 +2993,7 @@
         <v>116</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
     </row>
     <row r="9" spans="1:4" ht="300" x14ac:dyDescent="0.4">
@@ -3001,7 +3001,7 @@
         <v>117</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>167</v>
+        <v>352</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.4">
@@ -3014,7 +3014,7 @@
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A12" s="1" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="B12" s="1"/>
     </row>
@@ -3023,7 +3023,7 @@
         <v>116</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
     </row>
     <row r="14" spans="1:4" ht="300" x14ac:dyDescent="0.4">
@@ -3031,7 +3031,7 @@
         <v>117</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>166</v>
+        <v>354</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.4">
@@ -3044,7 +3044,7 @@
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A17" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.4">
@@ -3052,7 +3052,7 @@
         <v>116</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
     </row>
     <row r="19" spans="1:2" ht="225" x14ac:dyDescent="0.4">
@@ -3060,7 +3060,7 @@
         <v>117</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>191</v>
+        <v>353</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.4">
@@ -3068,7 +3068,7 @@
         <v>118</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>192</v>
+        <v>189</v>
       </c>
     </row>
   </sheetData>
@@ -3163,10 +3163,10 @@
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A6" s="1" t="s">
-        <v>193</v>
+        <v>190</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>194</v>
+        <v>191</v>
       </c>
       <c r="C6" s="1" t="s">
         <v>148</v>
@@ -3175,7 +3175,7 @@
         <v>130</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>195</v>
+        <v>192</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.4">
@@ -3226,7 +3226,7 @@
         <v>73</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>196</v>
+        <v>193</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.4">
@@ -3321,7 +3321,7 @@
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A17" s="1" t="s">
-        <v>197</v>
+        <v>194</v>
       </c>
       <c r="B17" s="1" t="s">
         <v>90</v>
@@ -3333,7 +3333,7 @@
         <v>148</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.4">
@@ -3350,7 +3350,7 @@
         <v>73</v>
       </c>
       <c r="E18" s="1" t="s">
-        <v>199</v>
+        <v>196</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.4">
@@ -3384,7 +3384,7 @@
         <v>73</v>
       </c>
       <c r="E20" s="1" t="s">
-        <v>207</v>
+        <v>204</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.4">
@@ -3406,7 +3406,7 @@
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A23" t="s">
-        <v>200</v>
+        <v>197</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.4">
@@ -3445,10 +3445,10 @@
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A26" s="1" t="s">
+        <v>198</v>
+      </c>
+      <c r="B26" s="1" t="s">
         <v>201</v>
-      </c>
-      <c r="B26" s="1" t="s">
-        <v>204</v>
       </c>
       <c r="C26" s="1" t="s">
         <v>130</v>
@@ -3457,15 +3457,15 @@
         <v>148</v>
       </c>
       <c r="E26" s="1" t="s">
-        <v>206</v>
+        <v>203</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A27" s="1" t="s">
-        <v>202</v>
+        <v>199</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>194</v>
+        <v>191</v>
       </c>
       <c r="C27" s="1" t="s">
         <v>72</v>
@@ -3474,15 +3474,15 @@
         <v>73</v>
       </c>
       <c r="E27" s="1" t="s">
-        <v>208</v>
+        <v>205</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A28" s="1" t="s">
-        <v>203</v>
+        <v>200</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>205</v>
+        <v>202</v>
       </c>
       <c r="C28" s="1" t="s">
         <v>130</v>
@@ -3518,10 +3518,10 @@
   <sheetData>
     <row r="2" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A2" s="1" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>209</v>
+        <v>206</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>110</v>
@@ -3530,10 +3530,10 @@
         <v>6</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>210</v>
+        <v>207</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>211</v>
+        <v>208</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.4">
@@ -3541,19 +3541,19 @@
         <v>1</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>212</v>
+        <v>209</v>
       </c>
       <c r="C3" s="1" t="s">
         <v>112</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>213</v>
+        <v>210</v>
       </c>
       <c r="E3" s="1" t="s">
         <v>31</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.4">
@@ -3561,19 +3561,19 @@
         <v>2</v>
       </c>
       <c r="B4" s="1" t="s">
+        <v>212</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>213</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>214</v>
+      </c>
+      <c r="E4" s="1" t="s">
         <v>215</v>
       </c>
-      <c r="C4" s="1" t="s">
+      <c r="F4" s="1" t="s">
         <v>216</v>
-      </c>
-      <c r="D4" s="1" t="s">
-        <v>217</v>
-      </c>
-      <c r="E4" s="1" t="s">
-        <v>218</v>
-      </c>
-      <c r="F4" s="1" t="s">
-        <v>219</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.4">
@@ -3581,19 +3581,19 @@
         <v>3</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>220</v>
+        <v>217</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>221</v>
+        <v>218</v>
       </c>
       <c r="E5" s="1" t="s">
         <v>111</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>222</v>
+        <v>219</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.4">
@@ -3601,19 +3601,19 @@
         <v>4</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="C6" s="1" t="s">
         <v>112</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>224</v>
+        <v>221</v>
       </c>
       <c r="E6" s="1" t="s">
         <v>31</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.4">
@@ -3621,19 +3621,19 @@
         <v>5</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>231</v>
+        <v>228</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="E7" s="1" t="s">
         <v>92</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.4">
@@ -3641,19 +3641,19 @@
         <v>6</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>228</v>
+        <v>225</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>230</v>
+        <v>227</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.4">
@@ -3661,7 +3661,7 @@
         <v>7</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>233</v>
+        <v>230</v>
       </c>
       <c r="C9" s="1" t="s">
         <v>112</v>
@@ -3673,7 +3673,7 @@
         <v>31</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>234</v>
+        <v>231</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.4">
@@ -3681,19 +3681,19 @@
         <v>8</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>235</v>
+        <v>232</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>312</v>
+        <v>309</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>313</v>
+        <v>310</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>314</v>
+        <v>311</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.4">
@@ -3701,19 +3701,19 @@
         <v>9</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>309</v>
+        <v>306</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>310</v>
+        <v>307</v>
       </c>
       <c r="E11" s="1" t="s">
         <v>125</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>234</v>
+        <v>231</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.4">
@@ -3721,19 +3721,19 @@
         <v>10</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>311</v>
+        <v>308</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>309</v>
+        <v>306</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>316</v>
+        <v>313</v>
       </c>
       <c r="E12" s="1" t="s">
         <v>125</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>234</v>
+        <v>231</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.4">
@@ -3741,19 +3741,19 @@
         <v>11</v>
       </c>
       <c r="B13" s="1" t="s">
+        <v>233</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>213</v>
+      </c>
+      <c r="D13" s="1" t="s">
+        <v>234</v>
+      </c>
+      <c r="E13" s="1" t="s">
+        <v>235</v>
+      </c>
+      <c r="F13" s="1" t="s">
         <v>236</v>
-      </c>
-      <c r="C13" s="1" t="s">
-        <v>216</v>
-      </c>
-      <c r="D13" s="1" t="s">
-        <v>237</v>
-      </c>
-      <c r="E13" s="1" t="s">
-        <v>238</v>
-      </c>
-      <c r="F13" s="1" t="s">
-        <v>239</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.4">
@@ -3761,19 +3761,19 @@
         <v>12</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>315</v>
+        <v>312</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>309</v>
+        <v>306</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>317</v>
+        <v>314</v>
       </c>
       <c r="E14" s="1" t="s">
         <v>125</v>
       </c>
       <c r="F14" s="1" t="s">
-        <v>318</v>
+        <v>315</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.4">
@@ -3781,19 +3781,19 @@
         <v>13</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>319</v>
+        <v>316</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>320</v>
+        <v>317</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>237</v>
+        <v>234</v>
       </c>
       <c r="E15" s="1" t="s">
         <v>125</v>
       </c>
       <c r="F15" s="1" t="s">
-        <v>318</v>
+        <v>315</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.4">
@@ -3801,19 +3801,19 @@
         <v>14</v>
       </c>
       <c r="B16" s="1" t="s">
+        <v>318</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>213</v>
+      </c>
+      <c r="D16" s="1" t="s">
+        <v>319</v>
+      </c>
+      <c r="E16" s="1" t="s">
+        <v>320</v>
+      </c>
+      <c r="F16" s="1" t="s">
         <v>321</v>
-      </c>
-      <c r="C16" s="1" t="s">
-        <v>216</v>
-      </c>
-      <c r="D16" s="1" t="s">
-        <v>322</v>
-      </c>
-      <c r="E16" s="1" t="s">
-        <v>323</v>
-      </c>
-      <c r="F16" s="1" t="s">
-        <v>324</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.4">
@@ -3821,19 +3821,19 @@
         <v>15</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>325</v>
+        <v>322</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>320</v>
+        <v>317</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>326</v>
+        <v>323</v>
       </c>
       <c r="E17" s="1" t="s">
         <v>125</v>
       </c>
       <c r="F17" s="1" t="s">
-        <v>327</v>
+        <v>324</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.4">
@@ -3841,19 +3841,19 @@
         <v>16</v>
       </c>
       <c r="B18" s="1" t="s">
+        <v>325</v>
+      </c>
+      <c r="C18" s="1" t="s">
+        <v>326</v>
+      </c>
+      <c r="D18" s="1" t="s">
+        <v>327</v>
+      </c>
+      <c r="E18" s="1" t="s">
         <v>328</v>
       </c>
-      <c r="C18" s="1" t="s">
+      <c r="F18" s="1" t="s">
         <v>329</v>
-      </c>
-      <c r="D18" s="1" t="s">
-        <v>330</v>
-      </c>
-      <c r="E18" s="1" t="s">
-        <v>331</v>
-      </c>
-      <c r="F18" s="1" t="s">
-        <v>332</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.4">
@@ -3861,19 +3861,19 @@
         <v>17</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>333</v>
+        <v>330</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>320</v>
+        <v>317</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>334</v>
+        <v>331</v>
       </c>
       <c r="E19" s="1" t="s">
         <v>125</v>
       </c>
       <c r="F19" s="1" t="s">
-        <v>335</v>
+        <v>332</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.4">
@@ -3881,19 +3881,19 @@
         <v>18</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>336</v>
+        <v>333</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>337</v>
+        <v>334</v>
       </c>
       <c r="E20" s="1" t="s">
-        <v>313</v>
+        <v>310</v>
       </c>
       <c r="F20" s="1" t="s">
-        <v>338</v>
+        <v>335</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.4">
@@ -3901,19 +3901,19 @@
         <v>19</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>339</v>
+        <v>336</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>309</v>
+        <v>306</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>340</v>
+        <v>337</v>
       </c>
       <c r="E21" s="1" t="s">
         <v>125</v>
       </c>
       <c r="F21" s="1" t="s">
-        <v>341</v>
+        <v>338</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.4">
@@ -3921,19 +3921,19 @@
         <v>20</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>342</v>
+        <v>339</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>237</v>
+        <v>234</v>
       </c>
       <c r="E22" s="1" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="F22" s="1" t="s">
-        <v>343</v>
+        <v>340</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.4">
@@ -3941,19 +3941,19 @@
         <v>21</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>344</v>
+        <v>341</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>320</v>
+        <v>317</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>345</v>
+        <v>342</v>
       </c>
       <c r="E23" s="1" t="s">
         <v>125</v>
       </c>
       <c r="F23" s="1" t="s">
-        <v>346</v>
+        <v>343</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.4">
@@ -3961,19 +3961,19 @@
         <v>22</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>347</v>
+        <v>344</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>320</v>
+        <v>317</v>
       </c>
       <c r="D24" s="1" t="s">
-        <v>348</v>
+        <v>345</v>
       </c>
       <c r="E24" s="1" t="s">
         <v>125</v>
       </c>
       <c r="F24" s="1" t="s">
-        <v>349</v>
+        <v>346</v>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.4">
@@ -3981,19 +3981,19 @@
         <v>23</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>350</v>
+        <v>347</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>309</v>
+        <v>306</v>
       </c>
       <c r="D25" s="1" t="s">
-        <v>351</v>
+        <v>348</v>
       </c>
       <c r="E25" s="1" t="s">
         <v>125</v>
       </c>
       <c r="F25" s="1" t="s">
-        <v>352</v>
+        <v>349</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.4">
@@ -4001,19 +4001,19 @@
         <v>24</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>353</v>
+        <v>350</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>320</v>
+        <v>317</v>
       </c>
       <c r="D26" s="1" t="s">
-        <v>354</v>
+        <v>351</v>
       </c>
       <c r="E26" s="1" t="s">
         <v>125</v>
       </c>
       <c r="F26" s="1" t="s">
-        <v>352</v>
+        <v>349</v>
       </c>
     </row>
   </sheetData>
@@ -4037,12 +4037,12 @@
   <sheetData>
     <row r="2" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
-        <v>240</v>
+        <v>237</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
-        <v>303</v>
+        <v>300</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.4">
@@ -4050,41 +4050,41 @@
         <v>0</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>242</v>
+        <v>239</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>243</v>
+        <v>240</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>244</v>
+        <v>241</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A5" s="1" t="s">
+        <v>242</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>243</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>244</v>
+      </c>
+      <c r="D5" s="1" t="s">
         <v>245</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>246</v>
-      </c>
-      <c r="C5" s="1" t="s">
-        <v>247</v>
-      </c>
-      <c r="D5" s="1" t="s">
-        <v>248</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A6" s="1" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>250</v>
+        <v>247</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>247</v>
+        <v>244</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>248</v>
+        <v>245</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.4">
@@ -4092,32 +4092,32 @@
         <v>115</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>251</v>
+        <v>248</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>252</v>
+        <v>249</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>253</v>
+        <v>250</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A8" s="1" t="s">
-        <v>254</v>
+        <v>251</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>255</v>
+        <v>252</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>256</v>
+        <v>253</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>248</v>
+        <v>245</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A10" t="s">
-        <v>306</v>
+        <v>303</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.4">
@@ -4125,88 +4125,88 @@
         <v>0</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>242</v>
+        <v>239</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>243</v>
+        <v>240</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>244</v>
+        <v>241</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A12" s="1" t="s">
-        <v>257</v>
+        <v>254</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>258</v>
+        <v>255</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>259</v>
+        <v>256</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>248</v>
+        <v>245</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A13" s="1" t="s">
-        <v>260</v>
+        <v>257</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>261</v>
+        <v>258</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>248</v>
+        <v>245</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A14" s="1" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>265</v>
+        <v>262</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>248</v>
+        <v>245</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A15" s="1" t="s">
-        <v>266</v>
+        <v>263</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>267</v>
+        <v>264</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>268</v>
+        <v>265</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>248</v>
+        <v>245</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A16" s="1" t="s">
-        <v>269</v>
+        <v>266</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>270</v>
+        <v>267</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>271</v>
+        <v>268</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>253</v>
+        <v>250</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A18" t="s">
-        <v>305</v>
+        <v>302</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.4">
@@ -4214,60 +4214,60 @@
         <v>0</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>242</v>
+        <v>239</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>243</v>
+        <v>240</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>244</v>
+        <v>241</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A20" s="1" t="s">
+        <v>269</v>
+      </c>
+      <c r="B20" s="1" t="s">
+        <v>270</v>
+      </c>
+      <c r="C20" s="1" t="s">
+        <v>271</v>
+      </c>
+      <c r="D20" s="1" t="s">
         <v>272</v>
-      </c>
-      <c r="B20" s="1" t="s">
-        <v>273</v>
-      </c>
-      <c r="C20" s="1" t="s">
-        <v>274</v>
-      </c>
-      <c r="D20" s="1" t="s">
-        <v>275</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A21" s="1" t="s">
+        <v>273</v>
+      </c>
+      <c r="B21" s="1" t="s">
+        <v>274</v>
+      </c>
+      <c r="C21" s="1" t="s">
+        <v>275</v>
+      </c>
+      <c r="D21" s="1" t="s">
         <v>276</v>
-      </c>
-      <c r="B21" s="1" t="s">
-        <v>277</v>
-      </c>
-      <c r="C21" s="1" t="s">
-        <v>278</v>
-      </c>
-      <c r="D21" s="1" t="s">
-        <v>279</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A22" s="1" t="s">
-        <v>280</v>
+        <v>277</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>281</v>
+        <v>278</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>282</v>
+        <v>279</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>279</v>
+        <v>276</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A24" t="s">
-        <v>304</v>
+        <v>301</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.4">
@@ -4275,65 +4275,65 @@
         <v>0</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>242</v>
+        <v>239</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>243</v>
+        <v>240</v>
       </c>
       <c r="D25" s="1" t="s">
-        <v>244</v>
+        <v>241</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A26" s="1" t="s">
-        <v>283</v>
+        <v>280</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>284</v>
+        <v>281</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>285</v>
+        <v>282</v>
       </c>
       <c r="D26" s="1" t="s">
-        <v>248</v>
+        <v>245</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A27" s="1" t="s">
-        <v>286</v>
+        <v>283</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>287</v>
+        <v>284</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>288</v>
+        <v>285</v>
       </c>
       <c r="D27" s="1" t="s">
-        <v>248</v>
+        <v>245</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A28" s="1" t="s">
-        <v>289</v>
+        <v>286</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>290</v>
+        <v>287</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>291</v>
+        <v>288</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>248</v>
+        <v>245</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A30" t="s">
-        <v>292</v>
+        <v>289</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A31" t="s">
-        <v>307</v>
+        <v>304</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.4">
@@ -4341,69 +4341,69 @@
         <v>0</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>242</v>
+        <v>239</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>243</v>
+        <v>240</v>
       </c>
       <c r="D32" s="1" t="s">
-        <v>244</v>
+        <v>241</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A33" s="1" t="s">
+        <v>290</v>
+      </c>
+      <c r="B33" s="1" t="s">
+        <v>291</v>
+      </c>
+      <c r="C33" s="1" t="s">
+        <v>292</v>
+      </c>
+      <c r="D33" s="1" t="s">
         <v>293</v>
-      </c>
-      <c r="B33" s="1" t="s">
-        <v>294</v>
-      </c>
-      <c r="C33" s="1" t="s">
-        <v>295</v>
-      </c>
-      <c r="D33" s="1" t="s">
-        <v>296</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A34" s="1" t="s">
-        <v>297</v>
+        <v>294</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>298</v>
+        <v>295</v>
       </c>
       <c r="C34" s="1" t="s">
-        <v>282</v>
+        <v>279</v>
       </c>
       <c r="D34" s="1" t="s">
-        <v>253</v>
+        <v>250</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A35" s="1" t="s">
-        <v>276</v>
+        <v>273</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>299</v>
+        <v>296</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>278</v>
+        <v>275</v>
       </c>
       <c r="D35" s="1" t="s">
-        <v>253</v>
+        <v>250</v>
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A36" s="1" t="s">
-        <v>300</v>
+        <v>297</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>301</v>
+        <v>298</v>
       </c>
       <c r="C36" s="1" t="s">
-        <v>302</v>
+        <v>299</v>
       </c>
       <c r="D36" s="1" t="s">
-        <v>253</v>
+        <v>250</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
delete old document and push new
</commit_message>
<xml_diff>
--- a/docs/仕様書.xlsx
+++ b/docs/仕様書.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\source\repos2\membership-management-system\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9ABA6045-5E22-494E-A73C-7B776B97382B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4DF460A8-31D9-473E-9D5A-A61E06C090F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-25545" yWindow="255" windowWidth="23505" windowHeight="13335" firstSheet="3" activeTab="7" xr2:uid="{B2A7CC7D-9061-4016-B10F-12143085F4DA}"/>
+    <workbookView xWindow="-25620" yWindow="3780" windowWidth="23505" windowHeight="9555" xr2:uid="{B2A7CC7D-9061-4016-B10F-12143085F4DA}"/>
   </bookViews>
   <sheets>
     <sheet name="01_システム概要" sheetId="1" r:id="rId1"/>
@@ -84,9 +84,6 @@
     <t>権限レベル</t>
   </si>
   <si>
-    <t>一般ユーザー / 管理者 / 上位管理者</t>
-  </si>
-  <si>
     <t>Python3 / Flask / MySQL / Railway / GitHub/ Jscode</t>
     <phoneticPr fontId="1"/>
   </si>
@@ -1670,6 +1667,16 @@
 またのご利用を心よりお待ちしております。
 あいうえお美術館会員管理システム
 noreply@oestemar-portfolio.xyz</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>一般ユーザー / 管理者 / 上位管理者/デモ用管理者</t>
+    <rPh sb="23" eb="24">
+      <t>ヨウ</t>
+    </rPh>
+    <rPh sb="24" eb="27">
+      <t>カンリシャ</t>
+    </rPh>
     <phoneticPr fontId="1"/>
   </si>
 </sst>
@@ -2127,7 +2134,7 @@
         <v>10</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="7" spans="1:2" ht="37.5" x14ac:dyDescent="0.4">
@@ -2135,7 +2142,7 @@
         <v>11</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.4">
@@ -2143,7 +2150,7 @@
         <v>12</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>13</v>
+        <v>354</v>
       </c>
     </row>
   </sheetData>
@@ -2167,315 +2174,315 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>19</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>20</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A2" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="B2" s="1" t="s">
         <v>123</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="C2" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="D2" s="1" t="s">
         <v>124</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>125</v>
       </c>
       <c r="E2" s="1"/>
       <c r="F2" s="1"/>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A3" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B3" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="C3" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="C3" s="1" t="s">
+      <c r="D3" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="D3" s="1" t="s">
+      <c r="E3" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="F3" s="1" t="s">
         <v>24</v>
-      </c>
-      <c r="E3" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="F3" s="1" t="s">
-        <v>25</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A4" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="B4" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="C4" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="D4" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="C4" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="D4" s="1" t="s">
+      <c r="E4" s="1" t="s">
         <v>28</v>
-      </c>
-      <c r="E4" s="1" t="s">
-        <v>29</v>
       </c>
       <c r="F4" s="1"/>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A5" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="B5" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="B5" s="1" t="s">
+      <c r="C5" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="D5" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="C5" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="D5" s="1" t="s">
-        <v>31</v>
-      </c>
       <c r="E5" s="1" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A6" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="B6" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="B6" s="1" t="s">
+      <c r="C6" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="D6" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="C6" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="D6" s="1" t="s">
-        <v>35</v>
-      </c>
       <c r="E6" s="1" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="F6" s="1"/>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A7" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="B7" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="B7" s="1" t="s">
+      <c r="C7" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="F7" s="1" t="s">
         <v>37</v>
-      </c>
-      <c r="C7" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="D7" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="E7" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="F7" s="1" t="s">
-        <v>38</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A8" s="1" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="B8" s="1" t="s">
+        <v>155</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="D8" s="1" t="s">
         <v>156</v>
       </c>
-      <c r="C8" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="D8" s="1" t="s">
-        <v>157</v>
-      </c>
       <c r="E8" s="1" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="F8" s="1"/>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A9" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="B9" s="1" t="s">
         <v>158</v>
       </c>
-      <c r="B9" s="1" t="s">
+      <c r="C9" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="D9" s="1" t="s">
         <v>159</v>
       </c>
-      <c r="C9" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="D9" s="1" t="s">
-        <v>160</v>
-      </c>
       <c r="E9" s="1" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="F9" s="1"/>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A10" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="B10" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="B10" s="1" t="s">
+      <c r="C10" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="C10" s="1" t="s">
-        <v>41</v>
-      </c>
       <c r="D10" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="F10" s="1"/>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A11" s="1" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="D11" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="E11" s="1" t="s">
+        <v>171</v>
+      </c>
+      <c r="F11" s="1" t="s">
         <v>127</v>
-      </c>
-      <c r="E11" s="1" t="s">
-        <v>172</v>
-      </c>
-      <c r="F11" s="1" t="s">
-        <v>128</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A12" s="1" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="F12" s="1"/>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A13" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="D13" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="E13" s="1" t="s">
+        <v>173</v>
+      </c>
+      <c r="F13" s="1" t="s">
         <v>42</v>
-      </c>
-      <c r="B13" s="1" t="s">
-        <v>113</v>
-      </c>
-      <c r="C13" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="D13" s="1" t="s">
-        <v>125</v>
-      </c>
-      <c r="E13" s="1" t="s">
-        <v>174</v>
-      </c>
-      <c r="F13" s="1" t="s">
-        <v>43</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A14" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="B14" s="1" t="s">
+        <v>141</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="D14" s="1" t="s">
         <v>140</v>
       </c>
-      <c r="B14" s="1" t="s">
-        <v>142</v>
-      </c>
-      <c r="C14" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="D14" s="1" t="s">
-        <v>141</v>
-      </c>
       <c r="E14" s="1" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="F14" s="1"/>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A15" s="1" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="E15" s="1" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="F15" s="1"/>
     </row>
     <row r="16" spans="1:6" ht="45" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A16" s="2" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="B16" s="1" t="s">
+        <v>166</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="D16" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="E16" s="2" t="s">
         <v>167</v>
-      </c>
-      <c r="C16" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="D16" s="1" t="s">
-        <v>139</v>
-      </c>
-      <c r="E16" s="2" t="s">
-        <v>168</v>
       </c>
       <c r="F16" s="1"/>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A17" s="1" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="B17" s="1"/>
       <c r="C17" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="F17" s="1"/>
     </row>
@@ -2499,241 +2506,241 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>45</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>46</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>8</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A2" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="B2" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="C2" s="1" t="s">
+        <v>177</v>
+      </c>
+      <c r="D2" s="1" t="s">
         <v>48</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>178</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>49</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A3" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="B3" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="C3" s="1" t="s">
+        <v>178</v>
+      </c>
+      <c r="D3" s="1" t="s">
         <v>51</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>179</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>52</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A4" s="1" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="D4" s="1"/>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A5" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="B5" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="B5" s="1" t="s">
-        <v>55</v>
-      </c>
       <c r="C5" s="1" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="D5" s="1"/>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A6" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="B6" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="B6" s="1" t="s">
-        <v>57</v>
-      </c>
       <c r="C6" s="1" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A7" s="1" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="D7" s="1"/>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A8" s="1" t="s">
+        <v>161</v>
+      </c>
+      <c r="B8" s="1" t="s">
         <v>162</v>
       </c>
-      <c r="B8" s="1" t="s">
-        <v>163</v>
-      </c>
       <c r="C8" s="1" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A9" s="1" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="D9" s="1"/>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A10" s="1" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="D10" s="1"/>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A11" s="1" t="s">
+        <v>135</v>
+      </c>
+      <c r="B11" s="1" t="s">
         <v>136</v>
       </c>
-      <c r="B11" s="1" t="s">
+      <c r="C11" s="1" t="s">
         <v>137</v>
-      </c>
-      <c r="C11" s="1" t="s">
-        <v>138</v>
       </c>
       <c r="D11" s="1"/>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A12" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="B12" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="B12" s="1" t="s">
-        <v>59</v>
-      </c>
       <c r="C12" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="D12" s="1"/>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A13" s="1" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D13" s="1"/>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A14" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="B14" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="B14" s="1" t="s">
-        <v>63</v>
-      </c>
       <c r="C14" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D14" s="1"/>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A15" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="B15" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="B15" s="1" t="s">
-        <v>65</v>
-      </c>
       <c r="C15" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D15" s="1"/>
     </row>
     <row r="16" spans="1:4" ht="56.25" x14ac:dyDescent="0.4">
       <c r="A16" s="1" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="B16" s="2" t="s">
+        <v>175</v>
+      </c>
+      <c r="C16" s="2" t="s">
         <v>176</v>
-      </c>
-      <c r="C16" s="2" t="s">
-        <v>177</v>
       </c>
       <c r="D16" s="1"/>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A17" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="B17" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="B17" s="1" t="s">
+      <c r="C17" s="1" t="s">
+        <v>163</v>
+      </c>
+      <c r="D17" s="1" t="s">
         <v>67</v>
-      </c>
-      <c r="C17" s="1" t="s">
-        <v>164</v>
-      </c>
-      <c r="D17" s="1" t="s">
-        <v>68</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A18" s="1" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="B18" s="1" t="s">
+        <v>151</v>
+      </c>
+      <c r="C18" s="1" t="s">
         <v>152</v>
-      </c>
-      <c r="C18" s="1" t="s">
-        <v>153</v>
       </c>
       <c r="D18" s="1"/>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A19" s="1" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="D19" s="1"/>
     </row>
@@ -2756,156 +2763,156 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>70</v>
-      </c>
       <c r="C1" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A2" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="B2" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="C2" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="C2" s="1" t="s">
-        <v>73</v>
-      </c>
       <c r="D2" s="1" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A3" s="1" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B3" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="C3" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="C3" s="1" t="s">
-        <v>73</v>
-      </c>
       <c r="D3" s="1" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A4" s="1" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A5" s="1" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A6" s="1" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A7" s="1" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A8" s="1" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A9" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A10" s="1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A11" s="1" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
     </row>
   </sheetData>
@@ -2927,148 +2934,148 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>76</v>
       </c>
-      <c r="C1" s="1" t="s">
-        <v>77</v>
-      </c>
       <c r="D1" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A2" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="B2" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="B2" s="1" t="s">
-        <v>79</v>
-      </c>
       <c r="C2" s="1" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A3" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="B3" s="1" t="s">
         <v>80</v>
       </c>
-      <c r="B3" s="1" t="s">
-        <v>81</v>
-      </c>
       <c r="C3" s="1" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D3" s="1"/>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A4" s="1" t="s">
+        <v>181</v>
+      </c>
+      <c r="B4" s="1" t="s">
         <v>182</v>
       </c>
-      <c r="B4" s="1" t="s">
-        <v>183</v>
-      </c>
       <c r="C4" s="1" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D4" s="1"/>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A6" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A7" s="1" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="B7" s="1"/>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A8" s="1" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
     </row>
     <row r="9" spans="1:4" ht="300" x14ac:dyDescent="0.4">
       <c r="A9" s="1" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A10" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="B10" s="1" t="s">
         <v>118</v>
-      </c>
-      <c r="B10" s="1" t="s">
-        <v>119</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A12" s="1" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="B12" s="1"/>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A13" s="1" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
     </row>
     <row r="14" spans="1:4" ht="300" x14ac:dyDescent="0.4">
       <c r="A14" s="1" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A15" s="1" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A17" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A18" s="1" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
     </row>
     <row r="19" spans="1:2" ht="225" x14ac:dyDescent="0.4">
       <c r="A19" s="1" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A20" s="1" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
     </row>
   </sheetData>
@@ -3090,408 +3097,408 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A1" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A2" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="B2" s="1" t="s">
         <v>82</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="C2" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="D2" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="D2" s="1" t="s">
-        <v>85</v>
-      </c>
       <c r="E2" s="1" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A3" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="B3" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="C3" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="E3" s="1" t="s">
         <v>87</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="E3" s="1" t="s">
-        <v>88</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A4" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="B4" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="C4" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="E4" s="1" t="s">
         <v>90</v>
-      </c>
-      <c r="C4" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="D4" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="E4" s="1" t="s">
-        <v>91</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A5" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="E5" s="1" t="s">
         <v>92</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>90</v>
-      </c>
-      <c r="C5" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="D5" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="E5" s="1" t="s">
-        <v>93</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A6" s="1" t="s">
+        <v>189</v>
+      </c>
+      <c r="B6" s="1" t="s">
         <v>190</v>
       </c>
-      <c r="B6" s="1" t="s">
+      <c r="C6" s="1" t="s">
+        <v>147</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="E6" s="1" t="s">
         <v>191</v>
-      </c>
-      <c r="C6" s="1" t="s">
-        <v>148</v>
-      </c>
-      <c r="D6" s="1" t="s">
-        <v>130</v>
-      </c>
-      <c r="E6" s="1" t="s">
-        <v>192</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A7" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>147</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="E7" s="1" t="s">
         <v>96</v>
-      </c>
-      <c r="B7" s="1" t="s">
-        <v>90</v>
-      </c>
-      <c r="C7" s="1" t="s">
-        <v>148</v>
-      </c>
-      <c r="D7" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="E7" s="1" t="s">
-        <v>97</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A8" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="E8" s="1" t="s">
         <v>98</v>
-      </c>
-      <c r="B8" s="1" t="s">
-        <v>90</v>
-      </c>
-      <c r="C8" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="D8" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="E8" s="1" t="s">
-        <v>99</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A9" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="B9" s="1" t="s">
         <v>100</v>
       </c>
-      <c r="B9" s="1" t="s">
-        <v>101</v>
-      </c>
       <c r="C9" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="D9" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="D9" s="1" t="s">
-        <v>73</v>
-      </c>
       <c r="E9" s="1" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A10" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="B10" s="1" t="s">
         <v>102</v>
       </c>
-      <c r="B10" s="1" t="s">
+      <c r="C10" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="E10" s="1" t="s">
         <v>103</v>
-      </c>
-      <c r="C10" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="D10" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="E10" s="1" t="s">
-        <v>104</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A11" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="E11" s="1" t="s">
         <v>105</v>
-      </c>
-      <c r="B11" s="1" t="s">
-        <v>103</v>
-      </c>
-      <c r="C11" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="D11" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="E11" s="1" t="s">
-        <v>106</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A12" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="E12" s="1" t="s">
         <v>94</v>
-      </c>
-      <c r="B12" s="1" t="s">
-        <v>90</v>
-      </c>
-      <c r="C12" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="D12" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="E12" s="1" t="s">
-        <v>95</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A14" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A15" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="B15" s="1" t="s">
         <v>82</v>
       </c>
-      <c r="B15" s="1" t="s">
+      <c r="C15" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="C15" s="1" t="s">
+      <c r="D15" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="D15" s="1" t="s">
-        <v>85</v>
-      </c>
       <c r="E15" s="1" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A16" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="B16" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="B16" s="1" t="s">
+      <c r="C16" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="D16" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="E16" s="1" t="s">
         <v>87</v>
-      </c>
-      <c r="C16" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="D16" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="E16" s="1" t="s">
-        <v>88</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A17" s="1" t="s">
+        <v>193</v>
+      </c>
+      <c r="B17" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="C17" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="D17" s="1" t="s">
+        <v>147</v>
+      </c>
+      <c r="E17" s="1" t="s">
         <v>194</v>
-      </c>
-      <c r="B17" s="1" t="s">
-        <v>90</v>
-      </c>
-      <c r="C17" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="D17" s="1" t="s">
-        <v>148</v>
-      </c>
-      <c r="E17" s="1" t="s">
-        <v>195</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A18" s="1" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="C18" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="D18" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="D18" s="1" t="s">
-        <v>73</v>
-      </c>
       <c r="E18" s="1" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A19" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="B19" s="1" t="s">
         <v>102</v>
       </c>
-      <c r="B19" s="1" t="s">
+      <c r="C19" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="D19" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="E19" s="1" t="s">
         <v>103</v>
-      </c>
-      <c r="C19" s="1" t="s">
-        <v>130</v>
-      </c>
-      <c r="D19" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="E19" s="1" t="s">
-        <v>104</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A20" s="1" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="E20" s="1" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A21" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="B21" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="C21" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="D21" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="E21" s="1" t="s">
         <v>94</v>
-      </c>
-      <c r="B21" s="1" t="s">
-        <v>90</v>
-      </c>
-      <c r="C21" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="D21" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="E21" s="1" t="s">
-        <v>95</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A23" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A24" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="B24" s="1" t="s">
         <v>82</v>
       </c>
-      <c r="B24" s="1" t="s">
+      <c r="C24" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="C24" s="1" t="s">
+      <c r="D24" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="D24" s="1" t="s">
-        <v>85</v>
-      </c>
       <c r="E24" s="1" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A25" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="B25" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="B25" s="1" t="s">
+      <c r="C25" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="D25" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="E25" s="1" t="s">
         <v>87</v>
-      </c>
-      <c r="C25" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="D25" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="E25" s="1" t="s">
-        <v>88</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A26" s="1" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="D26" s="1" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="E26" s="1" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A27" s="1" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="C27" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="D27" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="D27" s="1" t="s">
-        <v>73</v>
-      </c>
       <c r="E27" s="1" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A28" s="1" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="E28" s="1" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
   </sheetData>
@@ -3518,22 +3525,22 @@
   <sheetData>
     <row r="2" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A2" s="1" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="D2" s="1" t="s">
         <v>6</v>
       </c>
       <c r="E2" s="1" t="s">
+        <v>206</v>
+      </c>
+      <c r="F2" s="1" t="s">
         <v>207</v>
-      </c>
-      <c r="F2" s="1" t="s">
-        <v>208</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.4">
@@ -3541,19 +3548,19 @@
         <v>1</v>
       </c>
       <c r="B3" s="1" t="s">
+        <v>208</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="D3" s="1" t="s">
         <v>209</v>
       </c>
-      <c r="C3" s="1" t="s">
-        <v>112</v>
-      </c>
-      <c r="D3" s="1" t="s">
+      <c r="E3" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="F3" s="1" t="s">
         <v>210</v>
-      </c>
-      <c r="E3" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="F3" s="1" t="s">
-        <v>211</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.4">
@@ -3561,19 +3568,19 @@
         <v>2</v>
       </c>
       <c r="B4" s="1" t="s">
+        <v>211</v>
+      </c>
+      <c r="C4" s="1" t="s">
         <v>212</v>
       </c>
-      <c r="C4" s="1" t="s">
+      <c r="D4" s="1" t="s">
         <v>213</v>
       </c>
-      <c r="D4" s="1" t="s">
+      <c r="E4" s="1" t="s">
         <v>214</v>
       </c>
-      <c r="E4" s="1" t="s">
+      <c r="F4" s="1" t="s">
         <v>215</v>
-      </c>
-      <c r="F4" s="1" t="s">
-        <v>216</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.4">
@@ -3581,19 +3588,19 @@
         <v>3</v>
       </c>
       <c r="B5" s="1" t="s">
+        <v>216</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>212</v>
+      </c>
+      <c r="D5" s="1" t="s">
         <v>217</v>
       </c>
-      <c r="C5" s="1" t="s">
-        <v>213</v>
-      </c>
-      <c r="D5" s="1" t="s">
+      <c r="E5" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="F5" s="1" t="s">
         <v>218</v>
-      </c>
-      <c r="E5" s="1" t="s">
-        <v>111</v>
-      </c>
-      <c r="F5" s="1" t="s">
-        <v>219</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.4">
@@ -3601,19 +3608,19 @@
         <v>4</v>
       </c>
       <c r="B6" s="1" t="s">
+        <v>219</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="D6" s="1" t="s">
         <v>220</v>
       </c>
-      <c r="C6" s="1" t="s">
-        <v>112</v>
-      </c>
-      <c r="D6" s="1" t="s">
+      <c r="E6" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="F6" s="1" t="s">
         <v>221</v>
-      </c>
-      <c r="E6" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="F6" s="1" t="s">
-        <v>222</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.4">
@@ -3621,19 +3628,19 @@
         <v>5</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="D7" s="1" t="s">
+        <v>222</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="F7" s="1" t="s">
         <v>223</v>
-      </c>
-      <c r="E7" s="1" t="s">
-        <v>92</v>
-      </c>
-      <c r="F7" s="1" t="s">
-        <v>224</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.4">
@@ -3641,19 +3648,19 @@
         <v>6</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="D8" s="1" t="s">
+        <v>224</v>
+      </c>
+      <c r="E8" s="1" t="s">
         <v>225</v>
       </c>
-      <c r="E8" s="1" t="s">
+      <c r="F8" s="1" t="s">
         <v>226</v>
-      </c>
-      <c r="F8" s="1" t="s">
-        <v>227</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.4">
@@ -3661,19 +3668,19 @@
         <v>7</v>
       </c>
       <c r="B9" s="1" t="s">
+        <v>229</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="E9" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="F9" s="1" t="s">
         <v>230</v>
-      </c>
-      <c r="C9" s="1" t="s">
-        <v>112</v>
-      </c>
-      <c r="D9" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="E9" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="F9" s="1" t="s">
-        <v>231</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.4">
@@ -3681,19 +3688,19 @@
         <v>8</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="D10" s="1" t="s">
+        <v>308</v>
+      </c>
+      <c r="E10" s="1" t="s">
         <v>309</v>
       </c>
-      <c r="E10" s="1" t="s">
+      <c r="F10" s="1" t="s">
         <v>310</v>
-      </c>
-      <c r="F10" s="1" t="s">
-        <v>311</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.4">
@@ -3701,19 +3708,19 @@
         <v>9</v>
       </c>
       <c r="B11" s="1" t="s">
+        <v>304</v>
+      </c>
+      <c r="C11" s="1" t="s">
         <v>305</v>
       </c>
-      <c r="C11" s="1" t="s">
+      <c r="D11" s="1" t="s">
         <v>306</v>
       </c>
-      <c r="D11" s="1" t="s">
-        <v>307</v>
-      </c>
       <c r="E11" s="1" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.4">
@@ -3721,19 +3728,19 @@
         <v>10</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.4">
@@ -3741,19 +3748,19 @@
         <v>11</v>
       </c>
       <c r="B13" s="1" t="s">
+        <v>232</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>212</v>
+      </c>
+      <c r="D13" s="1" t="s">
         <v>233</v>
       </c>
-      <c r="C13" s="1" t="s">
-        <v>213</v>
-      </c>
-      <c r="D13" s="1" t="s">
+      <c r="E13" s="1" t="s">
         <v>234</v>
       </c>
-      <c r="E13" s="1" t="s">
+      <c r="F13" s="1" t="s">
         <v>235</v>
-      </c>
-      <c r="F13" s="1" t="s">
-        <v>236</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.4">
@@ -3761,19 +3768,19 @@
         <v>12</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="D14" s="1" t="s">
+        <v>313</v>
+      </c>
+      <c r="E14" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="F14" s="1" t="s">
         <v>314</v>
-      </c>
-      <c r="E14" s="1" t="s">
-        <v>125</v>
-      </c>
-      <c r="F14" s="1" t="s">
-        <v>315</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.4">
@@ -3781,19 +3788,19 @@
         <v>13</v>
       </c>
       <c r="B15" s="1" t="s">
+        <v>315</v>
+      </c>
+      <c r="C15" s="1" t="s">
         <v>316</v>
       </c>
-      <c r="C15" s="1" t="s">
-        <v>317</v>
-      </c>
       <c r="D15" s="1" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="E15" s="1" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="F15" s="1" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.4">
@@ -3801,19 +3808,19 @@
         <v>14</v>
       </c>
       <c r="B16" s="1" t="s">
+        <v>317</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>212</v>
+      </c>
+      <c r="D16" s="1" t="s">
         <v>318</v>
       </c>
-      <c r="C16" s="1" t="s">
-        <v>213</v>
-      </c>
-      <c r="D16" s="1" t="s">
+      <c r="E16" s="1" t="s">
         <v>319</v>
       </c>
-      <c r="E16" s="1" t="s">
+      <c r="F16" s="1" t="s">
         <v>320</v>
-      </c>
-      <c r="F16" s="1" t="s">
-        <v>321</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.4">
@@ -3821,19 +3828,19 @@
         <v>15</v>
       </c>
       <c r="B17" s="1" t="s">
+        <v>321</v>
+      </c>
+      <c r="C17" s="1" t="s">
+        <v>316</v>
+      </c>
+      <c r="D17" s="1" t="s">
         <v>322</v>
       </c>
-      <c r="C17" s="1" t="s">
-        <v>317</v>
-      </c>
-      <c r="D17" s="1" t="s">
+      <c r="E17" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="F17" s="1" t="s">
         <v>323</v>
-      </c>
-      <c r="E17" s="1" t="s">
-        <v>125</v>
-      </c>
-      <c r="F17" s="1" t="s">
-        <v>324</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.4">
@@ -3841,19 +3848,19 @@
         <v>16</v>
       </c>
       <c r="B18" s="1" t="s">
+        <v>324</v>
+      </c>
+      <c r="C18" s="1" t="s">
         <v>325</v>
       </c>
-      <c r="C18" s="1" t="s">
+      <c r="D18" s="1" t="s">
         <v>326</v>
       </c>
-      <c r="D18" s="1" t="s">
+      <c r="E18" s="1" t="s">
         <v>327</v>
       </c>
-      <c r="E18" s="1" t="s">
+      <c r="F18" s="1" t="s">
         <v>328</v>
-      </c>
-      <c r="F18" s="1" t="s">
-        <v>329</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.4">
@@ -3861,19 +3868,19 @@
         <v>17</v>
       </c>
       <c r="B19" s="1" t="s">
+        <v>329</v>
+      </c>
+      <c r="C19" s="1" t="s">
+        <v>316</v>
+      </c>
+      <c r="D19" s="1" t="s">
         <v>330</v>
       </c>
-      <c r="C19" s="1" t="s">
-        <v>317</v>
-      </c>
-      <c r="D19" s="1" t="s">
+      <c r="E19" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="F19" s="1" t="s">
         <v>331</v>
-      </c>
-      <c r="E19" s="1" t="s">
-        <v>125</v>
-      </c>
-      <c r="F19" s="1" t="s">
-        <v>332</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.4">
@@ -3881,19 +3888,19 @@
         <v>18</v>
       </c>
       <c r="B20" s="1" t="s">
+        <v>332</v>
+      </c>
+      <c r="C20" s="1" t="s">
+        <v>212</v>
+      </c>
+      <c r="D20" s="1" t="s">
         <v>333</v>
       </c>
-      <c r="C20" s="1" t="s">
-        <v>213</v>
-      </c>
-      <c r="D20" s="1" t="s">
+      <c r="E20" s="1" t="s">
+        <v>309</v>
+      </c>
+      <c r="F20" s="1" t="s">
         <v>334</v>
-      </c>
-      <c r="E20" s="1" t="s">
-        <v>310</v>
-      </c>
-      <c r="F20" s="1" t="s">
-        <v>335</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.4">
@@ -3901,19 +3908,19 @@
         <v>19</v>
       </c>
       <c r="B21" s="1" t="s">
+        <v>335</v>
+      </c>
+      <c r="C21" s="1" t="s">
+        <v>305</v>
+      </c>
+      <c r="D21" s="1" t="s">
         <v>336</v>
       </c>
-      <c r="C21" s="1" t="s">
-        <v>306</v>
-      </c>
-      <c r="D21" s="1" t="s">
+      <c r="E21" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="F21" s="1" t="s">
         <v>337</v>
-      </c>
-      <c r="E21" s="1" t="s">
-        <v>125</v>
-      </c>
-      <c r="F21" s="1" t="s">
-        <v>338</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.4">
@@ -3921,19 +3928,19 @@
         <v>20</v>
       </c>
       <c r="B22" s="1" t="s">
+        <v>338</v>
+      </c>
+      <c r="C22" s="1" t="s">
+        <v>212</v>
+      </c>
+      <c r="D22" s="1" t="s">
+        <v>233</v>
+      </c>
+      <c r="E22" s="1" t="s">
+        <v>234</v>
+      </c>
+      <c r="F22" s="1" t="s">
         <v>339</v>
-      </c>
-      <c r="C22" s="1" t="s">
-        <v>213</v>
-      </c>
-      <c r="D22" s="1" t="s">
-        <v>234</v>
-      </c>
-      <c r="E22" s="1" t="s">
-        <v>235</v>
-      </c>
-      <c r="F22" s="1" t="s">
-        <v>340</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.4">
@@ -3941,19 +3948,19 @@
         <v>21</v>
       </c>
       <c r="B23" s="1" t="s">
+        <v>340</v>
+      </c>
+      <c r="C23" s="1" t="s">
+        <v>316</v>
+      </c>
+      <c r="D23" s="1" t="s">
         <v>341</v>
       </c>
-      <c r="C23" s="1" t="s">
-        <v>317</v>
-      </c>
-      <c r="D23" s="1" t="s">
+      <c r="E23" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="F23" s="1" t="s">
         <v>342</v>
-      </c>
-      <c r="E23" s="1" t="s">
-        <v>125</v>
-      </c>
-      <c r="F23" s="1" t="s">
-        <v>343</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.4">
@@ -3961,19 +3968,19 @@
         <v>22</v>
       </c>
       <c r="B24" s="1" t="s">
+        <v>343</v>
+      </c>
+      <c r="C24" s="1" t="s">
+        <v>316</v>
+      </c>
+      <c r="D24" s="1" t="s">
         <v>344</v>
       </c>
-      <c r="C24" s="1" t="s">
-        <v>317</v>
-      </c>
-      <c r="D24" s="1" t="s">
+      <c r="E24" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="F24" s="1" t="s">
         <v>345</v>
-      </c>
-      <c r="E24" s="1" t="s">
-        <v>125</v>
-      </c>
-      <c r="F24" s="1" t="s">
-        <v>346</v>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.4">
@@ -3981,19 +3988,19 @@
         <v>23</v>
       </c>
       <c r="B25" s="1" t="s">
+        <v>346</v>
+      </c>
+      <c r="C25" s="1" t="s">
+        <v>305</v>
+      </c>
+      <c r="D25" s="1" t="s">
         <v>347</v>
       </c>
-      <c r="C25" s="1" t="s">
-        <v>306</v>
-      </c>
-      <c r="D25" s="1" t="s">
+      <c r="E25" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="F25" s="1" t="s">
         <v>348</v>
-      </c>
-      <c r="E25" s="1" t="s">
-        <v>125</v>
-      </c>
-      <c r="F25" s="1" t="s">
-        <v>349</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.4">
@@ -4001,19 +4008,19 @@
         <v>24</v>
       </c>
       <c r="B26" s="1" t="s">
+        <v>349</v>
+      </c>
+      <c r="C26" s="1" t="s">
+        <v>316</v>
+      </c>
+      <c r="D26" s="1" t="s">
         <v>350</v>
       </c>
-      <c r="C26" s="1" t="s">
-        <v>317</v>
-      </c>
-      <c r="D26" s="1" t="s">
-        <v>351</v>
-      </c>
       <c r="E26" s="1" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="F26" s="1" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
     </row>
   </sheetData>
@@ -4037,12 +4044,12 @@
   <sheetData>
     <row r="2" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.4">
@@ -4050,74 +4057,74 @@
         <v>0</v>
       </c>
       <c r="B4" s="1" t="s">
+        <v>238</v>
+      </c>
+      <c r="C4" s="1" t="s">
         <v>239</v>
       </c>
-      <c r="C4" s="1" t="s">
+      <c r="D4" s="1" t="s">
         <v>240</v>
-      </c>
-      <c r="D4" s="1" t="s">
-        <v>241</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A5" s="1" t="s">
+        <v>241</v>
+      </c>
+      <c r="B5" s="1" t="s">
         <v>242</v>
       </c>
-      <c r="B5" s="1" t="s">
+      <c r="C5" s="1" t="s">
         <v>243</v>
       </c>
-      <c r="C5" s="1" t="s">
+      <c r="D5" s="1" t="s">
         <v>244</v>
-      </c>
-      <c r="D5" s="1" t="s">
-        <v>245</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A6" s="1" t="s">
+        <v>245</v>
+      </c>
+      <c r="B6" s="1" t="s">
         <v>246</v>
       </c>
-      <c r="B6" s="1" t="s">
-        <v>247</v>
-      </c>
       <c r="C6" s="1" t="s">
+        <v>243</v>
+      </c>
+      <c r="D6" s="1" t="s">
         <v>244</v>
-      </c>
-      <c r="D6" s="1" t="s">
-        <v>245</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A7" s="1" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="B7" s="1" t="s">
+        <v>247</v>
+      </c>
+      <c r="C7" s="1" t="s">
         <v>248</v>
       </c>
-      <c r="C7" s="1" t="s">
+      <c r="D7" s="1" t="s">
         <v>249</v>
-      </c>
-      <c r="D7" s="1" t="s">
-        <v>250</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A8" s="1" t="s">
+        <v>250</v>
+      </c>
+      <c r="B8" s="1" t="s">
         <v>251</v>
       </c>
-      <c r="B8" s="1" t="s">
+      <c r="C8" s="1" t="s">
         <v>252</v>
       </c>
-      <c r="C8" s="1" t="s">
-        <v>253</v>
-      </c>
       <c r="D8" s="1" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A10" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.4">
@@ -4125,88 +4132,88 @@
         <v>0</v>
       </c>
       <c r="B11" s="1" t="s">
+        <v>238</v>
+      </c>
+      <c r="C11" s="1" t="s">
         <v>239</v>
       </c>
-      <c r="C11" s="1" t="s">
+      <c r="D11" s="1" t="s">
         <v>240</v>
-      </c>
-      <c r="D11" s="1" t="s">
-        <v>241</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A12" s="1" t="s">
+        <v>253</v>
+      </c>
+      <c r="B12" s="1" t="s">
         <v>254</v>
       </c>
-      <c r="B12" s="1" t="s">
+      <c r="C12" s="1" t="s">
         <v>255</v>
       </c>
-      <c r="C12" s="1" t="s">
-        <v>256</v>
-      </c>
       <c r="D12" s="1" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A13" s="1" t="s">
+        <v>256</v>
+      </c>
+      <c r="B13" s="1" t="s">
         <v>257</v>
       </c>
-      <c r="B13" s="1" t="s">
+      <c r="C13" s="1" t="s">
         <v>258</v>
       </c>
-      <c r="C13" s="1" t="s">
-        <v>259</v>
-      </c>
       <c r="D13" s="1" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A14" s="1" t="s">
+        <v>259</v>
+      </c>
+      <c r="B14" s="1" t="s">
         <v>260</v>
       </c>
-      <c r="B14" s="1" t="s">
+      <c r="C14" s="1" t="s">
         <v>261</v>
       </c>
-      <c r="C14" s="1" t="s">
-        <v>262</v>
-      </c>
       <c r="D14" s="1" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A15" s="1" t="s">
+        <v>262</v>
+      </c>
+      <c r="B15" s="1" t="s">
         <v>263</v>
       </c>
-      <c r="B15" s="1" t="s">
+      <c r="C15" s="1" t="s">
         <v>264</v>
       </c>
-      <c r="C15" s="1" t="s">
-        <v>265</v>
-      </c>
       <c r="D15" s="1" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A16" s="1" t="s">
+        <v>265</v>
+      </c>
+      <c r="B16" s="1" t="s">
         <v>266</v>
       </c>
-      <c r="B16" s="1" t="s">
+      <c r="C16" s="1" t="s">
         <v>267</v>
       </c>
-      <c r="C16" s="1" t="s">
-        <v>268</v>
-      </c>
       <c r="D16" s="1" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A18" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.4">
@@ -4214,60 +4221,60 @@
         <v>0</v>
       </c>
       <c r="B19" s="1" t="s">
+        <v>238</v>
+      </c>
+      <c r="C19" s="1" t="s">
         <v>239</v>
       </c>
-      <c r="C19" s="1" t="s">
+      <c r="D19" s="1" t="s">
         <v>240</v>
-      </c>
-      <c r="D19" s="1" t="s">
-        <v>241</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A20" s="1" t="s">
+        <v>268</v>
+      </c>
+      <c r="B20" s="1" t="s">
         <v>269</v>
       </c>
-      <c r="B20" s="1" t="s">
+      <c r="C20" s="1" t="s">
         <v>270</v>
       </c>
-      <c r="C20" s="1" t="s">
+      <c r="D20" s="1" t="s">
         <v>271</v>
-      </c>
-      <c r="D20" s="1" t="s">
-        <v>272</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A21" s="1" t="s">
+        <v>272</v>
+      </c>
+      <c r="B21" s="1" t="s">
         <v>273</v>
       </c>
-      <c r="B21" s="1" t="s">
+      <c r="C21" s="1" t="s">
         <v>274</v>
       </c>
-      <c r="C21" s="1" t="s">
+      <c r="D21" s="1" t="s">
         <v>275</v>
-      </c>
-      <c r="D21" s="1" t="s">
-        <v>276</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A22" s="1" t="s">
+        <v>276</v>
+      </c>
+      <c r="B22" s="1" t="s">
         <v>277</v>
       </c>
-      <c r="B22" s="1" t="s">
+      <c r="C22" s="1" t="s">
         <v>278</v>
       </c>
-      <c r="C22" s="1" t="s">
-        <v>279</v>
-      </c>
       <c r="D22" s="1" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A24" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.4">
@@ -4275,65 +4282,65 @@
         <v>0</v>
       </c>
       <c r="B25" s="1" t="s">
+        <v>238</v>
+      </c>
+      <c r="C25" s="1" t="s">
         <v>239</v>
       </c>
-      <c r="C25" s="1" t="s">
+      <c r="D25" s="1" t="s">
         <v>240</v>
-      </c>
-      <c r="D25" s="1" t="s">
-        <v>241</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A26" s="1" t="s">
+        <v>279</v>
+      </c>
+      <c r="B26" s="1" t="s">
         <v>280</v>
       </c>
-      <c r="B26" s="1" t="s">
+      <c r="C26" s="1" t="s">
         <v>281</v>
       </c>
-      <c r="C26" s="1" t="s">
-        <v>282</v>
-      </c>
       <c r="D26" s="1" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A27" s="1" t="s">
+        <v>282</v>
+      </c>
+      <c r="B27" s="1" t="s">
         <v>283</v>
       </c>
-      <c r="B27" s="1" t="s">
+      <c r="C27" s="1" t="s">
         <v>284</v>
       </c>
-      <c r="C27" s="1" t="s">
-        <v>285</v>
-      </c>
       <c r="D27" s="1" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A28" s="1" t="s">
+        <v>285</v>
+      </c>
+      <c r="B28" s="1" t="s">
         <v>286</v>
       </c>
-      <c r="B28" s="1" t="s">
+      <c r="C28" s="1" t="s">
         <v>287</v>
       </c>
-      <c r="C28" s="1" t="s">
-        <v>288</v>
-      </c>
       <c r="D28" s="1" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A30" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A31" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.4">
@@ -4341,69 +4348,69 @@
         <v>0</v>
       </c>
       <c r="B32" s="1" t="s">
+        <v>238</v>
+      </c>
+      <c r="C32" s="1" t="s">
         <v>239</v>
       </c>
-      <c r="C32" s="1" t="s">
+      <c r="D32" s="1" t="s">
         <v>240</v>
-      </c>
-      <c r="D32" s="1" t="s">
-        <v>241</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A33" s="1" t="s">
+        <v>289</v>
+      </c>
+      <c r="B33" s="1" t="s">
         <v>290</v>
       </c>
-      <c r="B33" s="1" t="s">
+      <c r="C33" s="1" t="s">
         <v>291</v>
       </c>
-      <c r="C33" s="1" t="s">
+      <c r="D33" s="1" t="s">
         <v>292</v>
-      </c>
-      <c r="D33" s="1" t="s">
-        <v>293</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A34" s="1" t="s">
+        <v>293</v>
+      </c>
+      <c r="B34" s="1" t="s">
         <v>294</v>
       </c>
-      <c r="B34" s="1" t="s">
-        <v>295</v>
-      </c>
       <c r="C34" s="1" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="D34" s="1" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A35" s="1" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="D35" s="1" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A36" s="1" t="s">
+        <v>296</v>
+      </c>
+      <c r="B36" s="1" t="s">
         <v>297</v>
       </c>
-      <c r="B36" s="1" t="s">
+      <c r="C36" s="1" t="s">
         <v>298</v>
       </c>
-      <c r="C36" s="1" t="s">
-        <v>299</v>
-      </c>
       <c r="D36" s="1" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
     </row>
   </sheetData>

</xml_diff>